<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-05-13 10:58:24
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -1030,7 +1030,11 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -1069,7 +1073,11 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-05-13 11:10:01
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -1032,10 +1032,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>1501</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1650</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -1075,10 +1079,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>1651</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card23 by admin at 2026-05-13 19:06:38
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -14164,7 +14164,11 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1501</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-05-15 18:30:32
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -1120,8 +1120,16 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1801</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card20 by admin at 2026-05-16 11:19:26
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -24504,15 +24504,31 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1238</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>16/5/2026</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card15 by admin at 2026-05-17 09:37:11
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -2158,7 +2158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3236,6 +3236,54 @@
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1253</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>17/5/2026</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card23 by admin at 2026-05-18 12:47:53
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -14140,15 +14140,31 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1283</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>18/5/2026</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card16 by admin at 2026-05-20 11:57:17
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -29858,15 +29858,31 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1162</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>20/5/2026</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 12:56:35
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13663,6 +13663,52 @@
           <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113640_2dc9d667.jpg,https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113558_f6dff8da.jpg</t>
         </is>
       </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>21/5/2026</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حسام،م.محمد عبدالله </t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:33:19
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13709,6 +13709,44 @@
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:35:16
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13742,7 +13742,11 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>21\5\2026</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:51:11
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13742,11 +13742,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>21\5\2026</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:51:17
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13747,6 +13747,44 @@
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:53:10
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13785,6 +13785,44 @@
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:55:27
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13823,6 +13823,44 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:55:45
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13861,6 +13861,44 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:56:20
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13899,6 +13899,44 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 16:56:30
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13937,6 +13937,44 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 17:20:36
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13975,6 +13975,44 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 17:20:49
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14013,6 +14013,44 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-05-21 17:20:56
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12641,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14051,6 +14051,44 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1275</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card4 by admin at 2026-05-21 17:24:18
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13716,26 +13716,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -13754,26 +13738,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -13792,26 +13760,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -13830,26 +13782,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -13868,26 +13804,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -13906,26 +13826,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -13944,26 +13848,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -13982,26 +13870,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
@@ -14020,26 +13892,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
@@ -14058,26 +13914,10 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>1151</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>1275</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card1 by admin at 2026-06-15 12:33:18
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -18525,7 +18525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19600,6 +19600,51 @@
           <t>م.صيام،م.عبدالله</t>
         </is>
       </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1260</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>19\5\2026</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-06-15 12:51:35
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -1130,8 +1130,16 @@
           <t>1950</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1888</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ث</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-06-15 12:53:00
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -1009,8 +1009,16 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-06-15 12:53:47
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -1009,16 +1009,8 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -1038,16 +1030,8 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1501</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1650</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -1085,16 +1069,8 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1651</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1800</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -1128,26 +1104,10 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>1801</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>1888</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>ث</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-06-15 12:58:09
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -978,7 +978,11 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1444</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-06-15 12:59:49
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -978,11 +978,7 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1444</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card9 by admin at 2026-06-16 20:38:20
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -9663,7 +9663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11123,6 +11123,48 @@
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1299</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>16/6//2026</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card21 by admin at 2026-06-17 12:58:40
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -23248,18 +23248,38 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1270</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>17/6/2026</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>حسام،ايهاب</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
تهيئة ورقة MachineData by admin at 2026-06-17 15:18:16
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -44,6 +44,7 @@
     <sheet name="TS-T5.1" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="TS-T5.2" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="BO-R" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="MachineData" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22796,6 +22797,47 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Card_Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Current_Tons</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Production_Speed_tons_per_hour</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Last_Update</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Last_Tons_Recorded</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
تهيئة ورقة ServiceLog by admin at 2026-06-17 15:18:18
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -45,6 +45,7 @@
     <sheet name="TS-T5.2" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="BO-R" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="MachineData" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="ServiceLog" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22838,6 +22839,57 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Card_Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Slice_Min_Tons</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Slice_Max_Tons</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Service_Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Execution_Date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Performed_By</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card3 by admin at 2026-06-18 09:47:07
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -17145,16 +17145,32 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1299</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>17/6/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>ايهاب</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
إضافة صف جديد في Card24 by admin at 2026-06-18 09:48:16
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2124,6 +2124,57 @@
       </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1295</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>17/6/2026</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>ايهاب</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card2 by admin at 2026-06-21 15:45:19
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -20233,18 +20233,34 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1298</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>21/6/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>ايهاب</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card11 by admin at 2026-06-22 17:45:39
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -7633,18 +7633,38 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1325</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>22/6/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ايهاب،حسام</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card15 by admin at 2026-06-28 08:41:17
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -2722,15 +2722,27 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1322</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>28/6/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card17 by admin at 2026-06-30 11:41:48
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -28770,7 +28770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29930,6 +29930,56 @@
           <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG-20260411-WA0022_1__a6dbf52b.jpg</t>
         </is>
       </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1267</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>25/5/2026</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>ايهاب</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card17 by admin at 2026-06-30 11:43:27
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -29229,15 +29229,27 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1324</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>30/6/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card17 by admin at 2026-06-30 11:44:06
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -29252,7 +29252,11 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>مصطفي</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
إضافة عمود جديد 'cylinder(0)' إلى Card4 by admin at 2026-07-01 06:31:01
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12744,7 +12744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12826,6 +12826,11 @@
       <c r="P1" t="inlineStr">
         <is>
           <t>Images</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>cylinder(0)</t>
         </is>
       </c>
     </row>
@@ -12858,6 +12863,7 @@
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -12904,6 +12910,7 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12934,6 +12941,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12980,6 +12988,7 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13022,6 +13031,7 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13072,6 +13082,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13122,6 +13133,7 @@
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13168,6 +13180,7 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13226,6 +13239,7 @@
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13284,6 +13298,7 @@
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13314,6 +13329,7 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13344,6 +13360,7 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13382,6 +13399,7 @@
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13420,6 +13438,7 @@
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13458,6 +13477,7 @@
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13496,6 +13516,7 @@
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13534,6 +13555,7 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13572,6 +13594,7 @@
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13610,6 +13633,7 @@
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13648,6 +13672,7 @@
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13686,6 +13711,7 @@
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13724,6 +13750,7 @@
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13766,6 +13793,7 @@
           <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113640_2dc9d667.jpg,https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113558_f6dff8da.jpg</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13812,6 +13840,7 @@
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13834,6 +13863,7 @@
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13856,6 +13886,7 @@
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13878,6 +13909,7 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13900,6 +13932,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13922,6 +13955,7 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13944,6 +13978,7 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13966,6 +14001,7 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13988,6 +14024,7 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14010,6 +14047,7 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14032,6 +14070,7 @@
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card4 by admin at 2026-07-02 09:50:21
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13316,7 +13316,11 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1333</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -13324,12 +13328,20 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2/7/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
إضافة صف جديد في Card2 by admin at 2026-07-04 12:22:09
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -19827,7 +19827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20909,6 +20909,43 @@
           <t>مصطفى ،عمر</t>
         </is>
       </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>7/5/2026</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card3 by admin at 2026-07-04 12:28:57
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -16802,7 +16802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17533,6 +17533,47 @@
           <t>تم سن فلاتس وتغير جريده خلفيه240,320</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>7/5/2026</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>ehab</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card18 by admin at 2026-07-06 12:51:30
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -27949,19 +27949,35 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1315</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>6/7/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
       <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card14 by admin at 2026-07-07 11:42:23
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -3836,18 +3836,38 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1343</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>7/7/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card5 by admin at 2026-07-08 11:57:15
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -16489,18 +16489,38 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1330</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>8/7/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>مصطفي.ايهاب</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card6 by admin at 2026-07-11 11:41:10
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -15684,17 +15684,33 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>6/6/2026</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>محمد عبدالله ،محمود ايهاب</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15712,7 +15728,11 @@
           <t>700</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>555</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -15720,10 +15740,18 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>11/7/2026</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>محمد عبدالله ،محمود ايهاب</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card6 by admin at 2026-07-11 11:42:09
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -15689,11 +15689,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -15734,7 +15730,11 @@
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card7 by admin at 2026-07-13 12:47:15
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12387,10 +12387,22 @@
           <t>700</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>556</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card7 by admin at 2026-07-13 12:51:25
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12325,13 +12325,25 @@
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>8/4/2026</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -12358,14 +12370,22 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>8/6/2026</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
@@ -12398,16 +12418,20 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>13/7/2026</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card6 by admin at 2026-07-14 09:14:58
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -15772,7 +15772,11 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card8 by admin at 2026-07-15 12:06:40
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -11839,15 +11839,31 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1344</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>15/7/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة عمود جديد 'cylinder(o)' إلى Card12 by admin at 2026-07-21 09:33:37
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5619,7 +5619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5701,6 +5701,11 @@
       <c r="P1" t="inlineStr">
         <is>
           <t>Images</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>cylinder(o)</t>
         </is>
       </c>
     </row>
@@ -5733,6 +5738,7 @@
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5779,6 +5785,7 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5809,6 +5816,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5855,6 +5863,7 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5897,6 +5906,7 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5947,6 +5957,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5993,6 +6004,7 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6039,6 +6051,7 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6101,6 +6114,7 @@
           <t>nan, IMG20251231154846_c9ad33b0.jpg, ٢٠٢٥_١٢_٣١_١٢_٠٦_٤٨_٣٣٧_d3c340d7.png, ٢٠٢٥_١٢_٣١_١٢_٠٦_٤٠_٤١٥_3f350cc1.png, Screenshot_٢٠٢٥-١٢-٣١-٠٩-٣٤-٢٦-٧٠_f2cb81fb7cf38af7978f186f2a61634a_ba293d6d.jpg, IMG20251229125736_58e0c250.jpg</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6159,6 +6173,7 @@
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6189,6 +6204,7 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6219,6 +6235,7 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6257,6 +6274,7 @@
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6295,6 +6313,7 @@
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6333,6 +6352,7 @@
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6371,6 +6391,7 @@
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6409,6 +6430,7 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6443,6 +6465,7 @@
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6477,6 +6500,7 @@
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6511,6 +6535,7 @@
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6553,6 +6578,7 @@
           <t>IMG-20251224-WA0078_4d39c8b8.jpg, IMG-20251224-WA0076_392f89a3.jpg, IMG-20251224-WA0074_1915b5cc.jpg, IMG-20251224-WA0068_8f71bcaa.jpg, IMG-20251224-WA0063_4029f5dc.jpg, IMG-20251224-WA0065_ee9e36a2.jpg, IMG-20251224-WA0061_5291e6be.jpg, IMG-20251224-WA0070_1da39212.jpg, IMG-20251224-WA0062_ba4b7fb3.jpg</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6587,6 +6613,7 @@
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6621,6 +6648,7 @@
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6655,6 +6683,7 @@
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6693,6 +6722,7 @@
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6731,6 +6761,7 @@
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6769,6 +6800,7 @@
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6807,6 +6839,7 @@
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6845,6 +6878,7 @@
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6883,6 +6917,7 @@
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6921,6 +6956,7 @@
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6959,6 +6995,7 @@
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6997,6 +7034,7 @@
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7035,6 +7073,7 @@
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7073,6 +7112,7 @@
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7112,6 +7152,7 @@
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة عمود جديد '1st licker in(o)' إلى Card12 by admin at 2026-07-21 09:34:04
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5619,7 +5619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5706,6 +5706,11 @@
       <c r="Q1" t="inlineStr">
         <is>
           <t>cylinder(o)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>1st licker in(o)</t>
         </is>
       </c>
     </row>
@@ -5739,6 +5744,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5786,6 +5792,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5817,6 +5824,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5864,6 +5872,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5907,6 +5916,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5958,6 +5968,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6005,6 +6016,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6052,6 +6064,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6115,6 +6128,7 @@
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6174,6 +6188,7 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6205,6 +6220,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6236,6 +6252,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6275,6 +6292,7 @@
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6314,6 +6332,7 @@
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6353,6 +6372,7 @@
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6392,6 +6412,7 @@
       </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6431,6 +6452,7 @@
       </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6466,6 +6488,7 @@
       </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6501,6 +6524,7 @@
       </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6536,6 +6560,7 @@
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6579,6 +6604,7 @@
         </is>
       </c>
       <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6614,6 +6640,7 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6649,6 +6676,7 @@
       </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6684,6 +6712,7 @@
       </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6723,6 +6752,7 @@
       </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6762,6 +6792,7 @@
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6801,6 +6832,7 @@
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6840,6 +6872,7 @@
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6879,6 +6912,7 @@
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6918,6 +6952,7 @@
       </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6957,6 +6992,7 @@
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6996,6 +7032,7 @@
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7035,6 +7072,7 @@
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7074,6 +7112,7 @@
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7113,6 +7152,7 @@
       </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7153,6 +7193,7 @@
       </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card12 by admin at 2026-07-21 09:35:21
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -6206,21 +6206,41 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1360</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>21/7/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card10 by admin at 2026-07-28 09:54:28
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -9093,15 +9093,31 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1363</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>28\7\2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card4 by admin at 2026-08-02 11:39:54
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13511,7 +13511,11 @@
           <t>1333</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1376</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -13556,8 +13560,16 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2/8/2026</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card4 by admin at 2026-08-02 11:41:21
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13511,11 +13511,7 @@
           <t>1333</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>1376</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -13560,16 +13556,8 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2/8/2026</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-08-02 11:41:53
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12934,7 +12934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14273,6 +14273,45 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1301</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1376</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card4 by admin at 2026-08-02 11:43:09
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -14306,7 +14306,11 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2/8/2026</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة عمود جديد 'cylinder(0)' إلى Card15 by admin at 2026-08-11 10:15:31
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -2187,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2279,6 +2279,11 @@
       <c r="R1" t="inlineStr">
         <is>
           <t>Serviced by.1</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>cylinder(0)</t>
         </is>
       </c>
     </row>
@@ -2325,6 +2330,7 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2357,6 +2363,7 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2405,6 +2412,7 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2445,6 +2453,7 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2489,6 +2498,7 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2533,6 +2543,7 @@
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2581,6 +2592,7 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2645,6 +2657,7 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2705,6 +2718,7 @@
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2749,6 +2763,7 @@
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2781,6 +2796,7 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2817,6 +2833,7 @@
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2853,6 +2870,7 @@
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2889,6 +2907,7 @@
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2925,6 +2944,7 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2965,6 +2985,7 @@
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3001,6 +3022,7 @@
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3037,6 +3059,7 @@
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3077,6 +3100,7 @@
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3117,6 +3141,7 @@
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3157,6 +3182,7 @@
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3197,6 +3223,7 @@
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3237,6 +3264,7 @@
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3277,6 +3305,7 @@
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3325,6 +3354,7 @@
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة عمود جديد '1st licker(0)' إلى Card15 by admin at 2026-08-11 10:15:57
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -2187,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:T26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2284,6 +2284,11 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>cylinder(0)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>1st licker(0)</t>
         </is>
       </c>
     </row>
@@ -2331,6 +2336,7 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2364,6 +2370,7 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2413,6 +2420,7 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2454,6 +2462,7 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2499,6 +2508,7 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2544,6 +2554,7 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2593,6 +2604,7 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2658,6 +2670,7 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2719,6 +2732,7 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2764,6 +2778,7 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2797,6 +2812,7 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2834,6 +2850,7 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2871,6 +2888,7 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2908,6 +2926,7 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2945,6 +2964,7 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2986,6 +3006,7 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3023,6 +3044,7 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3060,6 +3082,7 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3101,6 +3124,7 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3142,6 +3166,7 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3183,6 +3208,7 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3224,6 +3250,7 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3265,6 +3292,7 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3306,6 +3334,7 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3355,6 +3384,7 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card15 by admin at 2026-08-11 10:17:13
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -2187,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:T27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3385,6 +3385,56 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1301</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1398</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>11/8/2026</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card1 by admin at 2026-08-16 10:39:15
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -19759,15 +19759,27 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1413</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>16/8/2026</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card2 by admin at 2026-08-16 10:40:15
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -20809,15 +20809,27 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1397</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>16/8/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card3 by admin at 2026-08-17 11:23:04
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -17197,7 +17197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17969,6 +17969,47 @@
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1301</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1407</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>17/8/2026</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card16 by admin at 2026-08-18 12:45:46
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -31134,15 +31134,27 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1316</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>18/8/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card4 by admin at 2026-08-29 07:36:28
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -13044,7 +13044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14426,6 +14426,49 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1301</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1428</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>24/8/2026</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة عمود جديد 'cylinder(0)' إلى Card19 by admin at 2026-08-29 07:38:13
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -26979,7 +26979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27056,6 +27056,11 @@
       <c r="O1" t="inlineStr">
         <is>
           <t>Serviced by</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>cylinder(0)</t>
         </is>
       </c>
     </row>
@@ -27087,6 +27092,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -27124,6 +27130,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -27153,6 +27160,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -27182,6 +27190,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -27227,6 +27236,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -27268,6 +27278,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -27317,6 +27328,7 @@
           <t>م.محمد عبدالله ،تيم الكرد</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -27370,6 +27382,7 @@
           <t>م محمد عبدالله.محمود ايهاب</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -27399,6 +27412,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -27428,6 +27442,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -27457,6 +27472,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -27490,6 +27506,7 @@
           <t>تم العمل</t>
         </is>
       </c>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -27523,6 +27540,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -27556,6 +27574,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -27593,6 +27612,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -27630,6 +27650,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -27667,6 +27688,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -27704,6 +27726,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -27741,6 +27764,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -27778,6 +27802,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -27815,6 +27840,7 @@
           <t>م محمد عبدالله ،تيم الكرد</t>
         </is>
       </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -27852,6 +27878,7 @@
           <t>فني ورديه</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -27889,6 +27916,7 @@
           <t>سلامه و ناجي واسلام</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -27926,6 +27954,7 @@
           <t>رضا واسلام</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -27963,6 +27992,7 @@
           <t>سعيد</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة عمود جديد '1st licker in(o)' إلى Card19 by admin at 2026-08-29 07:38:26
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -26979,7 +26979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27061,6 +27061,11 @@
       <c r="P1" t="inlineStr">
         <is>
           <t>cylinder(0)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>1st licker in(o)</t>
         </is>
       </c>
     </row>
@@ -27093,6 +27098,7 @@
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -27131,6 +27137,7 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -27161,6 +27168,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -27191,6 +27199,7 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -27237,6 +27246,7 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -27279,6 +27289,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -27329,6 +27340,7 @@
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -27383,6 +27395,7 @@
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -27413,6 +27426,7 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -27443,6 +27457,7 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -27473,6 +27488,7 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -27507,6 +27523,7 @@
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -27541,6 +27558,7 @@
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -27575,6 +27593,7 @@
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -27613,6 +27632,7 @@
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -27651,6 +27671,7 @@
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -27689,6 +27710,7 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -27727,6 +27749,7 @@
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -27765,6 +27788,7 @@
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -27803,6 +27827,7 @@
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -27841,6 +27866,7 @@
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -27879,6 +27905,7 @@
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -27917,6 +27944,7 @@
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -27955,6 +27983,7 @@
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -27993,6 +28022,7 @@
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card19 by admin at 2026-08-29 07:39:25
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -27444,20 +27444,40 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1428</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>26/8/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card23 by admin at 2026-09-03 05:19:46
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -14992,15 +14992,27 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>30/8/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card12 by admin at 2026-09-06 11:33:13
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -6368,15 +6368,31 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1430</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>6/9/2026</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card16 by admin at 2026-09-06 11:35:04
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -30764,7 +30764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32267,6 +32267,49 @@
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1301</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1352</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>5/9/2026</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>